<commit_message>
Code is able to record real time timestamps of motor and speaker pulses
</commit_message>
<xml_diff>
--- a/Python Files/Summary Sheet.xlsx
+++ b/Python Files/Summary Sheet.xlsx
@@ -1,91 +1,33 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\uqtverga\Documents\Local Python Dev environment\QBI---Vibration-Box-10968-\Python Files\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BAAA026-643D-4679-983C-CAB12676F1E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Runs" sheetId="1" r:id="rId1"/>
+    <sheet name="Runs" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
-  <si>
-    <t>Timestamp</t>
-  </si>
-  <si>
-    <t>Recording Time (s)</t>
-  </si>
-  <si>
-    <t>Speaker</t>
-  </si>
-  <si>
-    <t>Speaker Freq (Hz)</t>
-  </si>
-  <si>
-    <t>Speaker On Time (s)</t>
-  </si>
-  <si>
-    <t>Speaker Off Time (s)</t>
-  </si>
-  <si>
-    <t>Camera</t>
-  </si>
-  <si>
-    <t>View Mode</t>
-  </si>
-  <si>
-    <t>Microphone</t>
-  </si>
-  <si>
-    <t>Motor</t>
-  </si>
-  <si>
-    <t>Motor Strength</t>
-  </si>
-  <si>
-    <t>Motor On Time (ms)</t>
-  </si>
-  <si>
-    <t>Motor Off Time (ms)</t>
-  </si>
-  <si>
-    <t>FLAC Out</t>
-  </si>
-  <si>
-    <t>h265 Out</t>
-  </si>
-  <si>
-    <t>MP4 Out</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -104,21 +46,80 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -406,58 +407,219 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:T2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29.140625" customWidth="1" min="7" max="7"/>
+    <col width="32.7109375" customWidth="1" min="8" max="8"/>
+    <col width="31.7109375" customWidth="1" min="9" max="9"/>
+    <col width="23.42578125" customWidth="1" min="10" max="10"/>
+    <col width="20.42578125" customWidth="1" min="11" max="11"/>
+    <col width="23.5703125" customWidth="1" min="12" max="12"/>
+    <col width="33" customWidth="1" min="13" max="13"/>
+    <col width="21.140625" customWidth="1" min="14" max="14"/>
+    <col width="22.5703125" customWidth="1" min="15" max="15"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Timestamp</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Recording Time (s)</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Speaker</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Speaker Freq (Hz)</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Speaker On Time (s)</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Speaker Off Time (s)</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Speaker Pulses (Real Time)</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Speaker Pulses (In Simulation time)</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Camera</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>View Mode</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Microphone</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Motor</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Motor Strength</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Motor On Time (ms)</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Motor Off Time (ms)</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>Motor Pulses (Real Time)</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>Motor Pulses (In Simulation time)</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>FLAC Out</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>h265 Out</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>MP4 Out</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>121502_08_07</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>61.5</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>250</v>
+      </c>
+      <c r="E2" t="n">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" t="s">
-        <v>13</v>
-      </c>
-      <c r="O1" t="s">
-        <v>14</v>
-      </c>
-      <c r="P1" t="s">
-        <v>15</v>
+      <c r="F2" t="n">
+        <v>19</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>12:15:02.879, 12:15:21.897, 12:15:40.937, 12:15:59.987</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>0.0, 19.02, 38.06, 57.11</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>12:15:06.629, 12:15:08.852, 12:15:11.033, 12:15:13.260, 12:15:15.433, 12:15:17.656, 12:15:19.834, 12:15:22.061, 12:15:24.235, 12:15:26.459, 12:15:28.680, 12:15:30.849, 12:15:33.070, 12:15:35.241, 12:15:37.463, 12:15:39.685, 12:15:41.853, 12:15:44.074, 12:15:46.246, 12:15:48.468, 12:15:50.690, 12:15:52.860, 12:15:55.081, 12:15:57.250, 12:15:59.470, 12:16:01.693, 12:16:03.863</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>3.75, 5.97, 8.16, 10.38, 12.55, 14.78, 16.96, 19.18, 21.36, 23.58, 25.8, 27.97, 30.19, 32.36, 34.59, 36.81, 38.98, 41.2, 43.37, 45.59, 47.81, 49.98, 52.2, 54.37, 56.59, 58.82, 60.99</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>